<commit_message>
Excel templates: Grott Luker brand band, Powered by BlueLine, disclaimers
- Every sheet opens with a navy band carrying the Grott Luker logo and
  "Powered by BlueLine Advisors".
- Read me sheets (and the Know Your Numbers page) close with About Grott
  Luker & Co., Powered by BlueLine Advisors (SEC disclosure, no advisory
  relationship), and the planning-record disclaimer; data and summary
  sheets carry the disclaimer under their totals.
- Workbook properties name both firms.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/GrottLuker-Know-Your-Numbers.xlsx
+++ b/public/templates/GrottLuker-Know-Your-Numbers.xlsx
@@ -19,13 +19,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0;($#,##0);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -75,12 +81,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF7D6"/>
+        <fgColor rgb="000F2440"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000F2440"/>
+        <fgColor rgb="00FFF7D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -115,22 +121,35 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -205,6 +224,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1171575" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -496,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -504,448 +553,498 @@
     <col width="50" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>POWERED BY  BLUELINE ADVISORS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Know Your Numbers</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>A one-page financial snapshot. Round numbers are fine — this is a conversation starter, not a tax return.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Grott Luker &amp; Co. · Client Decision Support Toolkit · platform by BlueLine Advisors</t>
-        </is>
-      </c>
-    </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Yellow cells are yours to fill in. White cells calculate themselves — leave them alone.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Assets</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Cash &amp; bank accounts</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="8" t="n"/>
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Investments (non-retirement)</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="8" t="n"/>
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="9" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Retirement accounts</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="8" t="n"/>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="9" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Real estate</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="8" t="n"/>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="9" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Business interests</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="8" t="n"/>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="9" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Personal property &amp; other</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="8" t="n"/>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="9" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Total assets</t>
         </is>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="11">
         <f>SUM(B7:B12)</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Liabilities</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Mortgage</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="8" t="n"/>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="9" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Auto loans</t>
         </is>
       </c>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="8" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="9" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Student loans</t>
         </is>
       </c>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="8" t="n"/>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="9" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Credit cards</t>
         </is>
       </c>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="8" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="9" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>Other debt</t>
         </is>
       </c>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="8" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="9" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>Total liabilities</t>
         </is>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="11">
         <f>SUM(B16:B20)</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Income</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Amount (per year)</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>Employment income</t>
         </is>
       </c>
-      <c r="B24" s="7" t="n"/>
-      <c r="C24" s="8" t="n"/>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="9" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Business / self-employment</t>
         </is>
       </c>
-      <c r="B25" s="7" t="n"/>
-      <c r="C25" s="8" t="n"/>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="9" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>Investment income</t>
         </is>
       </c>
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="8" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="9" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Other income</t>
         </is>
       </c>
-      <c r="B27" s="7" t="n"/>
-      <c r="C27" s="8" t="n"/>
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="9" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="inlineStr">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>Total income</t>
         </is>
       </c>
-      <c r="B28" s="10">
+      <c r="B28" s="11">
         <f>SUM(B24:B27)</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Expenses</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Amount (per year)</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>Housing</t>
         </is>
       </c>
-      <c r="B31" s="7" t="n"/>
-      <c r="C31" s="8" t="n"/>
+      <c r="B31" s="8" t="n"/>
+      <c r="C31" s="9" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>Living expenses</t>
         </is>
       </c>
-      <c r="B32" s="7" t="n"/>
-      <c r="C32" s="8" t="n"/>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="9" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>Debt payments</t>
         </is>
       </c>
-      <c r="B33" s="7" t="n"/>
-      <c r="C33" s="8" t="n"/>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="9" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>Other expenses</t>
         </is>
       </c>
-      <c r="B34" s="7" t="n"/>
-      <c r="C34" s="8" t="n"/>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="9" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="inlineStr">
+      <c r="A35" s="10" t="inlineStr">
         <is>
           <t>Total expenses</t>
         </is>
       </c>
-      <c r="B35" s="10">
+      <c r="B35" s="11">
         <f>SUM(B31:B34)</f>
         <v/>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>Other figures</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>Annual savings &amp; investing</t>
         </is>
       </c>
-      <c r="B38" s="7" t="n"/>
-      <c r="C38" s="8" t="n"/>
+      <c r="B38" s="8" t="n"/>
+      <c r="C38" s="9" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>Life insurance coverage</t>
         </is>
       </c>
-      <c r="B39" s="7" t="n"/>
-      <c r="C39" s="8" t="n"/>
+      <c r="B39" s="8" t="n"/>
+      <c r="C39" s="9" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
+      <c r="A40" s="7" t="inlineStr">
         <is>
           <t>Disability coverage (monthly benefit)</t>
         </is>
       </c>
-      <c r="B40" s="7" t="n"/>
-      <c r="C40" s="8" t="n"/>
+      <c r="B40" s="8" t="n"/>
+      <c r="C40" s="9" t="n"/>
     </row>
     <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>Your snapshot</t>
         </is>
       </c>
-      <c r="B42" s="5" t="inlineStr"/>
-      <c r="C42" s="5" t="inlineStr"/>
+      <c r="B42" s="6" t="inlineStr"/>
+      <c r="C42" s="6" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="9" t="inlineStr">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>Net worth</t>
         </is>
       </c>
-      <c r="B43" s="11">
+      <c r="B43" s="12">
         <f>B13-B21</f>
         <v/>
       </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="C43" s="13" t="inlineStr">
         <is>
           <t>assets − liabilities</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="9" t="inlineStr">
+      <c r="A44" s="10" t="inlineStr">
         <is>
           <t>Annual cash flow</t>
         </is>
       </c>
-      <c r="B44" s="11">
+      <c r="B44" s="12">
         <f>B28-B35</f>
         <v/>
       </c>
-      <c r="C44" s="3" t="inlineStr">
+      <c r="C44" s="13" t="inlineStr">
         <is>
           <t>income − expenses</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="9" t="inlineStr">
+      <c r="A45" s="10" t="inlineStr">
         <is>
           <t>Savings rate</t>
         </is>
       </c>
-      <c r="B45" s="12">
+      <c r="B45" s="14">
         <f>IF(B28&gt;0,B38/B28,0)</f>
         <v/>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C45" s="13" t="inlineStr">
         <is>
           <t>annual savings ÷ income</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="9" t="inlineStr">
+      <c r="A46" s="10" t="inlineStr">
         <is>
           <t>Debt-to-income</t>
         </is>
       </c>
-      <c r="B46" s="12">
+      <c r="B46" s="14">
         <f>IF(B28&gt;0,B33/B28,0)</f>
         <v/>
       </c>
-      <c r="C46" s="3" t="inlineStr">
+      <c r="C46" s="13" t="inlineStr">
         <is>
           <t>annual debt payments ÷ income</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>When you're done, send this file to Grott Luker &amp; Co. or type the figures into the online form at the link your CPA sent. Educational only; not tax, legal, or investment advice.</t>
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>When you are done, send this file to Grott Luker &amp; Co. or type the figures into the online form at the link your CPA sent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="16" customHeight="1">
+      <c r="A50" s="15" t="inlineStr">
+        <is>
+          <t>About Grott Luker &amp; Co.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="34" customHeight="1">
+      <c r="A51" s="16" t="inlineStr">
+        <is>
+          <t>Certified Public Accountants · Portsmouth, New Hampshire · Accounting | Tax Planning | Advisory. Questions about this log go to your Grott Luker CPA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="16" t="inlineStr"/>
+    </row>
+    <row r="53" ht="16" customHeight="1">
+      <c r="A53" s="15" t="inlineStr">
+        <is>
+          <t>Powered by BlueLine Advisors</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="50" customHeight="1">
+      <c r="A54" s="16" t="inlineStr">
+        <is>
+          <t>The Client Decision Support Toolkit and its templates are built and maintained by BlueLine Advisors, LLC, an SEC-registered investment adviser based in Exeter, NH (registration does not imply any particular level of skill). Using this workbook does not create an advisory relationship with BlueLine. blueline-advisors.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="16" customHeight="1">
+      <c r="A55" s="16" t="inlineStr"/>
+    </row>
+    <row r="56" ht="50" customHeight="1">
+      <c r="A56" s="17" t="inlineStr">
+        <is>
+          <t>Prepared with the Grott Luker &amp; Co. Client Decision Support Toolkit, powered by BlueLine Advisors. This workbook is an educational planning record, not tax, legal, accounting, or investment advice. Figures are the client’s own entries and should be reviewed by Grott Luker &amp; Co. before use in any return or decision.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:C1"/>
+  <mergeCells count="10">
+    <mergeCell ref="A56:C56"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="A55:C55"/>
+    <mergeCell ref="A50:C50"/>
     <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A54:C54"/>
     <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="A52:C52"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>